<commit_message>
Update question vault file and rename the link to it
</commit_message>
<xml_diff>
--- a/designer/client/src/assets/downloads/Question-vault.xlsx
+++ b/designer/client/src/assets/downloads/Question-vault.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30317"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://defra.sharepoint.com/teams/Team811/GOVUK/GOV.UK forms/Training and onboarding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBC88BFE-A2F7-4615-AFDC-F12387D8B86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00935868-0AD0-44D7-B94D-1E3C8BBA2EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="33975" yWindow="2415" windowWidth="20130" windowHeight="11535" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Standard questions " sheetId="1" r:id="rId1"/>
-    <sheet name="Example questions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
   <si>
     <t>Information type</t>
   </si>
@@ -45,16 +44,13 @@
     <t>Question</t>
   </si>
   <si>
-    <t>Short description recommendation</t>
+    <t>Recommended short description</t>
   </si>
   <si>
     <t>Optional hint text</t>
   </si>
   <si>
     <t>Guidance text</t>
-  </si>
-  <si>
-    <t>Answer limits</t>
   </si>
   <si>
     <r>
@@ -84,54 +80,28 @@
     <t xml:space="preserve">Name </t>
   </si>
   <si>
-    <t>What's your full name?</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>Enter your first and last name</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Do not add character limits to name fields 
-Asking for a full name is better than asking for first name and last name in separate boxes as not everyone has a name that fits nearly into that, for example because of cultural differences. In some cases they SME may ask for separate boxes so the answers given match how they have data stored in their records.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Should you ask for a full name?</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Think about the purpose of the form. For a form asking for a name purely as a way to contact a user, you wouldn't usually need to ask for a full name with  middle names. If it's more of a legal or formal submission you may need to ask for a full name.</t>
-    </r>
+    <t>What is your full name?</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hint text not usually needed, as the question is clear. 
+If you need someone's full legal name you might want to say 'Include any middle names'. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do not add character limits to name fields 
+Asking for a full name is better than asking for first name and last name in separate boxes as not everyone has a name that fits nearly into that, for example because of cultural differences. In some cases the subject matter expert (SME) may ask for separate boxes so the answers given match how they have data stored in their records, in which case you can be more flexible with this.
+Avoid asking users for their title. It’s extra work for them and you’re asking them to potentially reveal their gender and marital status, which they may not want to do. An SME may say title is needed becuase he has to appear on a legal document. In these cases you may have more justification to ask for it.  </t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>What's your email address?</t>
-  </si>
-  <si>
-    <t>email address</t>
+    <t>What is your email address?</t>
+  </si>
+  <si>
+    <t>Email address</t>
   </si>
   <si>
     <t>For example, ‘name@example.com’</t>
@@ -140,19 +110,16 @@
     <t>UK Address</t>
   </si>
   <si>
-    <t>What's your address?</t>
-  </si>
-  <si>
-    <t>address</t>
+    <t>What is your address?</t>
+  </si>
+  <si>
+    <t>Address</t>
   </si>
   <si>
     <t>Phone number</t>
   </si>
   <si>
-    <t>What's your phone number?</t>
-  </si>
-  <si>
-    <t>phone number</t>
+    <t>What is your phone number?</t>
   </si>
   <si>
     <t>This can be a landline or mobile number</t>
@@ -170,22 +137,31 @@
     <t xml:space="preserve">Issue date </t>
   </si>
   <si>
-    <t>For example, 01 01 2025 for 1 January 2025</t>
+    <t>For example, 1 1 2025 for 1 January 2025</t>
   </si>
   <si>
     <t xml:space="preserve">This shows users the format that's needed </t>
   </si>
   <si>
+    <t>Any question with a yes or no answer</t>
+  </si>
+  <si>
+    <t>For example: Do you like ice cream?</t>
+  </si>
+  <si>
+    <t>Do you like ice cream? (Use the full question as the short description to avoid a shorter version, for example 'Likes ice cream' looking like the answer is Y when the user might have answered N)</t>
+  </si>
+  <si>
     <t>CPH number</t>
   </si>
   <si>
-    <t>What's your county parish holding (CPH) number?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cph number </t>
-  </si>
-  <si>
-    <t>This is XXXX</t>
+    <t>What is your county parish holding (CPH) number?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPH number </t>
+  </si>
+  <si>
+    <t>This is a 9 digit number, for example: 12/123/1234</t>
   </si>
   <si>
     <t>^[0-9]{2}[ \/]?[0-9]{3}[ \/]?[0-9]{4}$</t>
@@ -194,10 +170,7 @@
     <t>SBI number</t>
   </si>
   <si>
-    <t>What's your single business indicator (SBI) number?</t>
-  </si>
-  <si>
-    <t>sbi number</t>
+    <t>What is your single business indicator (SBI) number?</t>
   </si>
   <si>
     <t>This is 9 digit number that starts with either a 1 or 2</t>
@@ -206,13 +179,13 @@
     <t>[1-2]\d{8}</t>
   </si>
   <si>
-    <t>FRN number</t>
-  </si>
-  <si>
-    <t>What's your XXXXXXX (FRN)?</t>
-  </si>
-  <si>
-    <t>frn number</t>
+    <t xml:space="preserve">CRN number </t>
+  </si>
+  <si>
+    <t>What is your customer reference number (CRN)?</t>
+  </si>
+  <si>
+    <t>CRN number</t>
   </si>
   <si>
     <t>This is a 10 digit number that starts with a 1</t>
@@ -221,19 +194,58 @@
     <t>1\d\d\d\d\d\d\d\d\d</t>
   </si>
   <si>
-    <t xml:space="preserve">CRN number </t>
-  </si>
-  <si>
-    <t>What's your customer reference number (CRN)?</t>
-  </si>
-  <si>
-    <t>crn number</t>
-  </si>
-  <si>
     <t xml:space="preserve">The 'add another' feature </t>
   </si>
   <si>
-    <t>Complete one page for each [species] that will be affected by the works. You can add more [species] on the next page.</t>
+    <t>Complete one page for each [species] that will be affected by the work. Add the first [species] on this page. If you need to, you can add more after selecting Continue.</t>
+  </si>
+  <si>
+    <t>Ordnance Survey (OS) grid reference</t>
+  </si>
+  <si>
+    <t>What is your Ordnance Survey (OS) grid reference?</t>
+  </si>
+  <si>
+    <t>Do not use 'National Grid reference number'. Use the map component.</t>
+  </si>
+  <si>
+    <t>Any other information (asked right at the end of a form)</t>
+  </si>
+  <si>
+    <t>Do you have any more relevant information to give?</t>
+  </si>
+  <si>
+    <t>This could be, for example XXX (get the SME to give a couple of examples of things they may need to see that haven't been ask for elsewhere)</t>
+  </si>
+  <si>
+    <t>Preferred language (this will always be context dependent within a form, but it gives some ideas and preferences)</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Use 'give' instead of 'provide'</t>
+  </si>
+  <si>
+    <t>It's plainer English</t>
+  </si>
+  <si>
+    <t>Do not use 'please' or 'sorry'</t>
+  </si>
+  <si>
+    <t>These are not used on GOV.UK</t>
+  </si>
+  <si>
+    <t>Use 'Upload...'</t>
+  </si>
+  <si>
+    <t>This makes it clear that user needs to use the upload feature to give this</t>
+  </si>
+  <si>
+    <t>Use 'explain' or 'tell us' but use one consistently</t>
   </si>
 </sst>
 </file>
@@ -280,14 +292,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -300,8 +311,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -337,11 +354,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -367,6 +434,47 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -702,19 +810,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N49"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:M43"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="44.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="31" style="1" customWidth="1"/>
-    <col min="4" max="5" width="32.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="25.85546875" customWidth="1"/>
-    <col min="7" max="7" width="41.5703125" customWidth="1"/>
-    <col min="8" max="8" width="59.42578125" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" customWidth="1"/>
+    <col min="7" max="7" width="71.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="48">
+    <row r="1" spans="1:13" ht="47.1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -730,619 +838,524 @@
       <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-    </row>
-    <row r="2" spans="1:14" ht="204" customHeight="1">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:13" ht="184.5" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="9" t="s">
+      <c r="G2" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="30">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" s="2" t="s">
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:14" ht="30">
-      <c r="A5" s="2" t="s">
+    </row>
+    <row r="5" spans="1:13" ht="29.1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
+      <c r="G5" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="29.1">
+      <c r="A6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="30">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2" t="s">
+      <c r="G6" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="102.75" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+    </row>
+    <row r="8" spans="1:13" ht="29.1">
+      <c r="A8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="E8" s="3"/>
-      <c r="F8" s="2"/>
+      <c r="F8" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+    </row>
+    <row r="9" spans="1:13" ht="29.1">
+      <c r="A9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>38</v>
+      </c>
       <c r="E9" s="3"/>
-      <c r="F9" s="2"/>
+      <c r="F9" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:14" ht="30">
-      <c r="A10" s="2" t="s">
-        <v>30</v>
+    </row>
+    <row r="10" spans="1:13" ht="29.1">
+      <c r="A10" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E10" s="3"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:14" ht="30">
-      <c r="A11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:14" ht="30">
-      <c r="A12" s="2" t="s">
-        <v>40</v>
+      <c r="F10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" ht="84.75" customHeight="1">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="22"/>
+    </row>
+    <row r="12" spans="1:13" ht="29.1">
+      <c r="A12" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:14" ht="30">
-      <c r="A13" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="57.95">
+      <c r="A13" s="3" t="s">
+        <v>50</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="5"/>
+        <v>51</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="23"/>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="20"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" spans="1:14" ht="60">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6"/>
+    </row>
+    <row r="15" spans="1:13" ht="30.75" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="10"/>
+    </row>
+    <row r="16" spans="1:13" ht="20.25" customHeight="1">
+      <c r="A16" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>57</v>
+      </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6"/>
+    </row>
+    <row r="19" spans="1:7" ht="29.1">
+      <c r="A19" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>61</v>
+      </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="5"/>
+    </row>
+    <row r="20" spans="1:7" ht="29.1">
+      <c r="A20" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" s="5"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="5"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="5"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="5"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="5"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="5"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="5"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" s="5"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="5"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="5"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="5"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="5"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-    </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="5"/>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="5"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="5"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="5"/>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="5"/>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="5"/>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="5"/>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="5"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="5"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="5"/>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="5"/>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="5"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="5"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="5"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="5"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="5"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" s="5"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D49654A-0481-4907-AA2F-B4FE8ED423FE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <mergeCells count="1">
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="d1117845-93f6-4da3-abaa-fcb4fa669c78" ContentTypeId="0x010100A5BF1C78D9F64B679A5EBDE1C6598EBC01" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Defra document" ma:contentTypeID="0x010100A5BF1C78D9F64B679A5EBDE1C6598EBC01003D2B3DC3CBDAFE41BB43F5029A3739DC" ma:contentTypeVersion="32" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8f60470352fd9f9ea0e1988685f8c7fd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="662745e8-e224-48e8-a2e3-254862b8c2f5" xmlns:ns3="425b2036-7ca2-443f-9b95-8f1f612e0310" xmlns:ns4="916594dc-a2f1-4535-a0f4-a83afd51207d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cde55e1b5a06f85c92df71cc22b807a1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1742,7 +1755,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lae2bfa7b6474897ab4a53f76ea236c7 xmlns="662745e8-e224-48e8-a2e3-254862b8c2f5">
@@ -1821,7 +1834,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -1871,22 +1884,36 @@
 </spe:Receivers>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="d1117845-93f6-4da3-abaa-fcb4fa669c78" ContentTypeId="0x010100A5BF1C78D9F64B679A5EBDE1C6598EBC01" PreviousValue="false"/>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACA1887B-5466-436C-A9FB-7070320131DF}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D0687ED-4D9A-4827-902F-8B5BACF8F0BC}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7420430C-00C9-4BF2-97F1-A03698ACEC53}"/>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B08A4546-6E6C-40EB-8A7F-5EBBEA82094D}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFC778C2-7034-49E3-9906-F4E90209CCF9}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACA1887B-5466-436C-A9FB-7070320131DF}"/>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D0687ED-4D9A-4827-902F-8B5BACF8F0BC}"/>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7420430C-00C9-4BF2-97F1-A03698ACEC53}"/>
 </file>
</xml_diff>

<commit_message>
DF-1179 resources url (#1528)
* Fix question protocol spreadsheet download link

* Update question vault file and rename the link to it
</commit_message>
<xml_diff>
--- a/designer/client/src/assets/downloads/Question-vault.xlsx
+++ b/designer/client/src/assets/downloads/Question-vault.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30317"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://defra.sharepoint.com/teams/Team811/GOVUK/GOV.UK forms/Training and onboarding/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBC88BFE-A2F7-4615-AFDC-F12387D8B86B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{00935868-0AD0-44D7-B94D-1E3C8BBA2EB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="33975" yWindow="2415" windowWidth="20130" windowHeight="11535" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Standard questions " sheetId="1" r:id="rId1"/>
-    <sheet name="Example questions" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="63">
   <si>
     <t>Information type</t>
   </si>
@@ -45,16 +44,13 @@
     <t>Question</t>
   </si>
   <si>
-    <t>Short description recommendation</t>
+    <t>Recommended short description</t>
   </si>
   <si>
     <t>Optional hint text</t>
   </si>
   <si>
     <t>Guidance text</t>
-  </si>
-  <si>
-    <t>Answer limits</t>
   </si>
   <si>
     <r>
@@ -84,54 +80,28 @@
     <t xml:space="preserve">Name </t>
   </si>
   <si>
-    <t>What's your full name?</t>
-  </si>
-  <si>
-    <t>name</t>
-  </si>
-  <si>
-    <t>Enter your first and last name</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Do not add character limits to name fields 
-Asking for a full name is better than asking for first name and last name in separate boxes as not everyone has a name that fits nearly into that, for example because of cultural differences. In some cases they SME may ask for separate boxes so the answers given match how they have data stored in their records.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Should you ask for a full name?</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Think about the purpose of the form. For a form asking for a name purely as a way to contact a user, you wouldn't usually need to ask for a full name with  middle names. If it's more of a legal or formal submission you may need to ask for a full name.</t>
-    </r>
+    <t>What is your full name?</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hint text not usually needed, as the question is clear. 
+If you need someone's full legal name you might want to say 'Include any middle names'. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Do not add character limits to name fields 
+Asking for a full name is better than asking for first name and last name in separate boxes as not everyone has a name that fits nearly into that, for example because of cultural differences. In some cases the subject matter expert (SME) may ask for separate boxes so the answers given match how they have data stored in their records, in which case you can be more flexible with this.
+Avoid asking users for their title. It’s extra work for them and you’re asking them to potentially reveal their gender and marital status, which they may not want to do. An SME may say title is needed becuase he has to appear on a legal document. In these cases you may have more justification to ask for it.  </t>
   </si>
   <si>
     <t>Email</t>
   </si>
   <si>
-    <t>What's your email address?</t>
-  </si>
-  <si>
-    <t>email address</t>
+    <t>What is your email address?</t>
+  </si>
+  <si>
+    <t>Email address</t>
   </si>
   <si>
     <t>For example, ‘name@example.com’</t>
@@ -140,19 +110,16 @@
     <t>UK Address</t>
   </si>
   <si>
-    <t>What's your address?</t>
-  </si>
-  <si>
-    <t>address</t>
+    <t>What is your address?</t>
+  </si>
+  <si>
+    <t>Address</t>
   </si>
   <si>
     <t>Phone number</t>
   </si>
   <si>
-    <t>What's your phone number?</t>
-  </si>
-  <si>
-    <t>phone number</t>
+    <t>What is your phone number?</t>
   </si>
   <si>
     <t>This can be a landline or mobile number</t>
@@ -170,22 +137,31 @@
     <t xml:space="preserve">Issue date </t>
   </si>
   <si>
-    <t>For example, 01 01 2025 for 1 January 2025</t>
+    <t>For example, 1 1 2025 for 1 January 2025</t>
   </si>
   <si>
     <t xml:space="preserve">This shows users the format that's needed </t>
   </si>
   <si>
+    <t>Any question with a yes or no answer</t>
+  </si>
+  <si>
+    <t>For example: Do you like ice cream?</t>
+  </si>
+  <si>
+    <t>Do you like ice cream? (Use the full question as the short description to avoid a shorter version, for example 'Likes ice cream' looking like the answer is Y when the user might have answered N)</t>
+  </si>
+  <si>
     <t>CPH number</t>
   </si>
   <si>
-    <t>What's your county parish holding (CPH) number?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cph number </t>
-  </si>
-  <si>
-    <t>This is XXXX</t>
+    <t>What is your county parish holding (CPH) number?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CPH number </t>
+  </si>
+  <si>
+    <t>This is a 9 digit number, for example: 12/123/1234</t>
   </si>
   <si>
     <t>^[0-9]{2}[ \/]?[0-9]{3}[ \/]?[0-9]{4}$</t>
@@ -194,10 +170,7 @@
     <t>SBI number</t>
   </si>
   <si>
-    <t>What's your single business indicator (SBI) number?</t>
-  </si>
-  <si>
-    <t>sbi number</t>
+    <t>What is your single business indicator (SBI) number?</t>
   </si>
   <si>
     <t>This is 9 digit number that starts with either a 1 or 2</t>
@@ -206,13 +179,13 @@
     <t>[1-2]\d{8}</t>
   </si>
   <si>
-    <t>FRN number</t>
-  </si>
-  <si>
-    <t>What's your XXXXXXX (FRN)?</t>
-  </si>
-  <si>
-    <t>frn number</t>
+    <t xml:space="preserve">CRN number </t>
+  </si>
+  <si>
+    <t>What is your customer reference number (CRN)?</t>
+  </si>
+  <si>
+    <t>CRN number</t>
   </si>
   <si>
     <t>This is a 10 digit number that starts with a 1</t>
@@ -221,19 +194,58 @@
     <t>1\d\d\d\d\d\d\d\d\d</t>
   </si>
   <si>
-    <t xml:space="preserve">CRN number </t>
-  </si>
-  <si>
-    <t>What's your customer reference number (CRN)?</t>
-  </si>
-  <si>
-    <t>crn number</t>
-  </si>
-  <si>
     <t xml:space="preserve">The 'add another' feature </t>
   </si>
   <si>
-    <t>Complete one page for each [species] that will be affected by the works. You can add more [species] on the next page.</t>
+    <t>Complete one page for each [species] that will be affected by the work. Add the first [species] on this page. If you need to, you can add more after selecting Continue.</t>
+  </si>
+  <si>
+    <t>Ordnance Survey (OS) grid reference</t>
+  </si>
+  <si>
+    <t>What is your Ordnance Survey (OS) grid reference?</t>
+  </si>
+  <si>
+    <t>Do not use 'National Grid reference number'. Use the map component.</t>
+  </si>
+  <si>
+    <t>Any other information (asked right at the end of a form)</t>
+  </si>
+  <si>
+    <t>Do you have any more relevant information to give?</t>
+  </si>
+  <si>
+    <t>This could be, for example XXX (get the SME to give a couple of examples of things they may need to see that haven't been ask for elsewhere)</t>
+  </si>
+  <si>
+    <t>Preferred language (this will always be context dependent within a form, but it gives some ideas and preferences)</t>
+  </si>
+  <si>
+    <t>Term</t>
+  </si>
+  <si>
+    <t>Reason</t>
+  </si>
+  <si>
+    <t>Use 'give' instead of 'provide'</t>
+  </si>
+  <si>
+    <t>It's plainer English</t>
+  </si>
+  <si>
+    <t>Do not use 'please' or 'sorry'</t>
+  </si>
+  <si>
+    <t>These are not used on GOV.UK</t>
+  </si>
+  <si>
+    <t>Use 'Upload...'</t>
+  </si>
+  <si>
+    <t>This makes it clear that user needs to use the upload feature to give this</t>
+  </si>
+  <si>
+    <t>Use 'explain' or 'tell us' but use one consistently</t>
   </si>
 </sst>
 </file>
@@ -280,14 +292,13 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -300,8 +311,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -337,11 +354,61 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -367,6 +434,47 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -702,19 +810,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:N49"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
+  <dimension ref="A1:M43"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="30.7109375" customWidth="1"/>
-    <col min="2" max="2" width="44.85546875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.85546875" style="1" customWidth="1"/>
     <col min="3" max="3" width="31" style="1" customWidth="1"/>
-    <col min="4" max="5" width="32.28515625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="25.85546875" customWidth="1"/>
-    <col min="7" max="7" width="41.5703125" customWidth="1"/>
-    <col min="8" max="8" width="59.42578125" customWidth="1"/>
+    <col min="4" max="4" width="32.28515625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="41.5703125" customWidth="1"/>
+    <col min="7" max="7" width="71.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="48">
+    <row r="1" spans="1:13" ht="47.1">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -730,619 +838,524 @@
       <c r="E1" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
-        <v>7</v>
-      </c>
+      <c r="H1" s="1"/>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
       <c r="M1" s="1"/>
-      <c r="N1" s="1"/>
-    </row>
-    <row r="2" spans="1:14" ht="204" customHeight="1">
-      <c r="A2" s="2" t="s">
+    </row>
+    <row r="2" spans="1:13" ht="184.5" customHeight="1">
+      <c r="A2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>10</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>11</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="9" t="s">
+      <c r="G2" s="9" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13">
+      <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" ht="30">
-      <c r="A3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>15</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>16</v>
       </c>
       <c r="E3" s="3"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-    </row>
-    <row r="4" spans="1:14">
-      <c r="A4" s="2" t="s">
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-    </row>
-    <row r="5" spans="1:14" ht="30">
-      <c r="A5" s="2" t="s">
+    </row>
+    <row r="5" spans="1:13" ht="29.1">
+      <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
       </c>
       <c r="E5" s="3"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2" t="s">
+      <c r="G5" s="2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="29.1">
+      <c r="A6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" ht="30">
-      <c r="A6" s="2" t="s">
+      <c r="C6" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D6" s="3" t="s">
         <v>26</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2" t="s">
+      <c r="G6" s="2" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="102.75" customHeight="1">
+      <c r="A7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="7" spans="1:14">
-      <c r="A7" s="2"/>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
+      <c r="C7" s="3" t="s">
+        <v>30</v>
+      </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-    </row>
-    <row r="8" spans="1:14">
-      <c r="A8" s="2"/>
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
+    </row>
+    <row r="8" spans="1:13" ht="29.1">
+      <c r="A8" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>34</v>
+      </c>
       <c r="E8" s="3"/>
-      <c r="F8" s="2"/>
+      <c r="F8" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-    </row>
-    <row r="9" spans="1:14">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
+    </row>
+    <row r="9" spans="1:13" ht="29.1">
+      <c r="A9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>38</v>
+      </c>
       <c r="E9" s="3"/>
-      <c r="F9" s="2"/>
+      <c r="F9" s="4" t="s">
+        <v>39</v>
+      </c>
       <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-    </row>
-    <row r="10" spans="1:14" ht="30">
-      <c r="A10" s="2" t="s">
-        <v>30</v>
+    </row>
+    <row r="10" spans="1:13" ht="29.1">
+      <c r="A10" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E10" s="3"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H10" s="2"/>
-    </row>
-    <row r="11" spans="1:14" ht="30">
-      <c r="A11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="3"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="H11" s="2"/>
-    </row>
-    <row r="12" spans="1:14" ht="30">
-      <c r="A12" s="2" t="s">
-        <v>40</v>
+      <c r="F10" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:13" ht="84.75" customHeight="1">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="5"/>
+      <c r="G11" s="22"/>
+    </row>
+    <row r="12" spans="1:13" ht="29.1">
+      <c r="A12" s="3" t="s">
+        <v>47</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H12" s="2"/>
-    </row>
-    <row r="13" spans="1:14" ht="30">
-      <c r="A13" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
+      </c>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="5" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="13" spans="1:13" ht="57.95">
+      <c r="A13" s="3" t="s">
+        <v>50</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="3"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="H13" s="2"/>
-    </row>
-    <row r="14" spans="1:14">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="5"/>
+        <v>51</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="5"/>
+      <c r="G13" s="23"/>
+    </row>
+    <row r="14" spans="1:13">
+      <c r="A14" s="17"/>
+      <c r="B14" s="18"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="20"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
-    </row>
-    <row r="15" spans="1:14">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
-    </row>
-    <row r="16" spans="1:14" ht="60">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="5"/>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6"/>
+    </row>
+    <row r="15" spans="1:13" ht="30.75" customHeight="1">
+      <c r="A15" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="B15" s="25"/>
+      <c r="C15" s="25"/>
+      <c r="D15" s="25"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="10"/>
+    </row>
+    <row r="16" spans="1:13" ht="20.25" customHeight="1">
+      <c r="A16" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="10"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>57</v>
+      </c>
       <c r="C17" s="6"/>
       <c r="D17" s="6"/>
       <c r="E17" s="6"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="5"/>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="5"/>
-      <c r="B18" s="6"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>59</v>
+      </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
       <c r="E18" s="6"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="5"/>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6"/>
+    </row>
+    <row r="19" spans="1:7" ht="29.1">
+      <c r="A19" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>61</v>
+      </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="5"/>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="5"/>
+    </row>
+    <row r="20" spans="1:7" ht="29.1">
+      <c r="A20" s="6" t="s">
+        <v>62</v>
+      </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="5"/>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" s="5"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="6"/>
       <c r="B21" s="6"/>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
       <c r="E21" s="6"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="5"/>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" s="5"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="6"/>
       <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="5"/>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" s="5"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="6"/>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="5"/>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" s="5"/>
+    </row>
+    <row r="24" spans="1:7">
+      <c r="A24" s="6"/>
       <c r="B24" s="6"/>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" s="5"/>
+    </row>
+    <row r="25" spans="1:7">
+      <c r="A25" s="6"/>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
       <c r="E25" s="6"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="5"/>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" s="5"/>
+    </row>
+    <row r="26" spans="1:7">
+      <c r="A26" s="6"/>
       <c r="B26" s="6"/>
       <c r="C26" s="6"/>
       <c r="D26" s="6"/>
       <c r="E26" s="6"/>
       <c r="F26" s="5"/>
       <c r="G26" s="5"/>
-      <c r="H26" s="5"/>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" s="5"/>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" s="6"/>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
       <c r="D27" s="6"/>
       <c r="E27" s="6"/>
       <c r="F27" s="5"/>
       <c r="G27" s="5"/>
-      <c r="H27" s="5"/>
-    </row>
-    <row r="28" spans="1:8">
-      <c r="A28" s="5"/>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" s="6"/>
       <c r="B28" s="6"/>
       <c r="C28" s="6"/>
       <c r="D28" s="6"/>
       <c r="E28" s="6"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-    </row>
-    <row r="29" spans="1:8">
-      <c r="A29" s="5"/>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" s="6"/>
       <c r="B29" s="6"/>
       <c r="C29" s="6"/>
       <c r="D29" s="6"/>
       <c r="E29" s="6"/>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
-      <c r="H29" s="5"/>
-    </row>
-    <row r="30" spans="1:8">
-      <c r="A30" s="5"/>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" s="6"/>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
       <c r="D30" s="6"/>
       <c r="E30" s="6"/>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
-      <c r="H30" s="5"/>
-    </row>
-    <row r="31" spans="1:8">
-      <c r="A31" s="5"/>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" s="6"/>
       <c r="B31" s="6"/>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
       <c r="E31" s="6"/>
       <c r="F31" s="5"/>
       <c r="G31" s="5"/>
-      <c r="H31" s="5"/>
-    </row>
-    <row r="32" spans="1:8">
-      <c r="A32" s="5"/>
+    </row>
+    <row r="32" spans="1:7">
+      <c r="A32" s="6"/>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
       <c r="D32" s="6"/>
       <c r="E32" s="6"/>
       <c r="F32" s="5"/>
       <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-    </row>
-    <row r="33" spans="1:8">
-      <c r="A33" s="5"/>
+    </row>
+    <row r="33" spans="1:7">
+      <c r="A33" s="6"/>
       <c r="B33" s="6"/>
       <c r="C33" s="6"/>
       <c r="D33" s="6"/>
       <c r="E33" s="6"/>
       <c r="F33" s="5"/>
       <c r="G33" s="5"/>
-      <c r="H33" s="5"/>
-    </row>
-    <row r="34" spans="1:8">
-      <c r="A34" s="5"/>
+    </row>
+    <row r="34" spans="1:7">
+      <c r="A34" s="6"/>
       <c r="B34" s="6"/>
       <c r="C34" s="6"/>
       <c r="D34" s="6"/>
       <c r="E34" s="6"/>
       <c r="F34" s="5"/>
       <c r="G34" s="5"/>
-      <c r="H34" s="5"/>
-    </row>
-    <row r="35" spans="1:8">
-      <c r="A35" s="5"/>
+    </row>
+    <row r="35" spans="1:7">
+      <c r="A35" s="6"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
       <c r="D35" s="6"/>
       <c r="E35" s="6"/>
       <c r="F35" s="5"/>
       <c r="G35" s="5"/>
-      <c r="H35" s="5"/>
-    </row>
-    <row r="36" spans="1:8">
-      <c r="A36" s="5"/>
+    </row>
+    <row r="36" spans="1:7">
+      <c r="A36" s="6"/>
       <c r="B36" s="6"/>
       <c r="C36" s="6"/>
       <c r="D36" s="6"/>
       <c r="E36" s="6"/>
       <c r="F36" s="5"/>
       <c r="G36" s="5"/>
-      <c r="H36" s="5"/>
-    </row>
-    <row r="37" spans="1:8">
-      <c r="A37" s="5"/>
+    </row>
+    <row r="37" spans="1:7">
+      <c r="A37" s="6"/>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
       <c r="D37" s="6"/>
       <c r="E37" s="6"/>
       <c r="F37" s="5"/>
       <c r="G37" s="5"/>
-      <c r="H37" s="5"/>
-    </row>
-    <row r="38" spans="1:8">
-      <c r="A38" s="5"/>
+    </row>
+    <row r="38" spans="1:7">
+      <c r="A38" s="6"/>
       <c r="B38" s="6"/>
       <c r="C38" s="6"/>
       <c r="D38" s="6"/>
       <c r="E38" s="6"/>
       <c r="F38" s="5"/>
       <c r="G38" s="5"/>
-      <c r="H38" s="5"/>
-    </row>
-    <row r="39" spans="1:8">
-      <c r="A39" s="5"/>
+    </row>
+    <row r="39" spans="1:7">
+      <c r="A39" s="6"/>
       <c r="B39" s="6"/>
       <c r="C39" s="6"/>
       <c r="D39" s="6"/>
       <c r="E39" s="6"/>
       <c r="F39" s="5"/>
       <c r="G39" s="5"/>
-      <c r="H39" s="5"/>
-    </row>
-    <row r="40" spans="1:8">
-      <c r="A40" s="5"/>
+    </row>
+    <row r="40" spans="1:7">
+      <c r="A40" s="6"/>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
       <c r="D40" s="6"/>
       <c r="E40" s="6"/>
       <c r="F40" s="5"/>
       <c r="G40" s="5"/>
-      <c r="H40" s="5"/>
-    </row>
-    <row r="41" spans="1:8">
-      <c r="A41" s="5"/>
+    </row>
+    <row r="41" spans="1:7">
+      <c r="A41" s="6"/>
       <c r="B41" s="6"/>
       <c r="C41" s="6"/>
       <c r="D41" s="6"/>
       <c r="E41" s="6"/>
       <c r="F41" s="5"/>
       <c r="G41" s="5"/>
-      <c r="H41" s="5"/>
-    </row>
-    <row r="42" spans="1:8">
-      <c r="A42" s="5"/>
+    </row>
+    <row r="42" spans="1:7">
+      <c r="A42" s="6"/>
       <c r="B42" s="6"/>
       <c r="C42" s="6"/>
       <c r="D42" s="6"/>
       <c r="E42" s="6"/>
       <c r="F42" s="5"/>
       <c r="G42" s="5"/>
-      <c r="H42" s="5"/>
-    </row>
-    <row r="43" spans="1:8">
-      <c r="A43" s="5"/>
+    </row>
+    <row r="43" spans="1:7">
+      <c r="A43" s="6"/>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
       <c r="D43" s="6"/>
       <c r="E43" s="6"/>
       <c r="F43" s="5"/>
       <c r="G43" s="5"/>
-      <c r="H43" s="5"/>
-    </row>
-    <row r="44" spans="1:8">
-      <c r="A44" s="5"/>
-      <c r="B44" s="6"/>
-      <c r="C44" s="6"/>
-      <c r="D44" s="6"/>
-      <c r="E44" s="6"/>
-      <c r="F44" s="5"/>
-      <c r="G44" s="5"/>
-      <c r="H44" s="5"/>
-    </row>
-    <row r="45" spans="1:8">
-      <c r="A45" s="5"/>
-      <c r="B45" s="6"/>
-      <c r="C45" s="6"/>
-      <c r="D45" s="6"/>
-      <c r="E45" s="6"/>
-      <c r="F45" s="5"/>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-    </row>
-    <row r="46" spans="1:8">
-      <c r="A46" s="5"/>
-      <c r="B46" s="6"/>
-      <c r="C46" s="6"/>
-      <c r="D46" s="6"/>
-      <c r="E46" s="6"/>
-      <c r="F46" s="5"/>
-      <c r="G46" s="5"/>
-      <c r="H46" s="5"/>
-    </row>
-    <row r="47" spans="1:8">
-      <c r="A47" s="5"/>
-      <c r="B47" s="6"/>
-      <c r="C47" s="6"/>
-      <c r="D47" s="6"/>
-      <c r="E47" s="6"/>
-      <c r="F47" s="5"/>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
-    </row>
-    <row r="48" spans="1:8">
-      <c r="A48" s="5"/>
-      <c r="B48" s="6"/>
-      <c r="C48" s="6"/>
-      <c r="D48" s="6"/>
-      <c r="E48" s="6"/>
-      <c r="F48" s="5"/>
-      <c r="G48" s="5"/>
-      <c r="H48" s="5"/>
-    </row>
-    <row r="49" spans="1:8">
-      <c r="A49" s="5"/>
-      <c r="B49" s="6"/>
-      <c r="C49" s="6"/>
-      <c r="D49" s="6"/>
-      <c r="E49" s="6"/>
-      <c r="F49" s="5"/>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D49654A-0481-4907-AA2F-B4FE8ED423FE}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData/>
+  <mergeCells count="1">
+    <mergeCell ref="A15:F15"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="d1117845-93f6-4da3-abaa-fcb4fa669c78" ContentTypeId="0x010100A5BF1C78D9F64B679A5EBDE1C6598EBC01" PreviousValue="false"/>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Defra document" ma:contentTypeID="0x010100A5BF1C78D9F64B679A5EBDE1C6598EBC01003D2B3DC3CBDAFE41BB43F5029A3739DC" ma:contentTypeVersion="32" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8f60470352fd9f9ea0e1988685f8c7fd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="662745e8-e224-48e8-a2e3-254862b8c2f5" xmlns:ns3="425b2036-7ca2-443f-9b95-8f1f612e0310" xmlns:ns4="916594dc-a2f1-4535-a0f4-a83afd51207d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="cde55e1b5a06f85c92df71cc22b807a1" ns1:_="" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1742,7 +1755,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lae2bfa7b6474897ab4a53f76ea236c7 xmlns="662745e8-e224-48e8-a2e3-254862b8c2f5">
@@ -1821,7 +1834,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <spe:Receivers xmlns:spe="http://schemas.microsoft.com/sharepoint/events">
   <Receiver>
@@ -1871,22 +1884,36 @@
 </spe:Receivers>
 </file>
 
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item5.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="d1117845-93f6-4da3-abaa-fcb4fa669c78" ContentTypeId="0x010100A5BF1C78D9F64B679A5EBDE1C6598EBC01" PreviousValue="false"/>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACA1887B-5466-436C-A9FB-7070320131DF}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D0687ED-4D9A-4827-902F-8B5BACF8F0BC}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7420430C-00C9-4BF2-97F1-A03698ACEC53}"/>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B08A4546-6E6C-40EB-8A7F-5EBBEA82094D}"/>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFC778C2-7034-49E3-9906-F4E90209CCF9}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ACA1887B-5466-436C-A9FB-7070320131DF}"/>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5D0687ED-4D9A-4827-902F-8B5BACF8F0BC}"/>
-</file>
-
-<file path=customXml/itemProps5.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7420430C-00C9-4BF2-97F1-A03698ACEC53}"/>
 </file>
</xml_diff>